<commit_message>
rename OREXlsxConverter to OREBuilder & add functionality to pass in a dictionary of portfolio instead of excel file & cleanup
</commit_message>
<xml_diff>
--- a/ORELab/templates/sample_trades.xlsx
+++ b/ORELab/templates/sample_trades.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hieunguyen/Downloads/projects/ORE/ORELab/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{115A356B-24A4-0A4C-B4E6-9AFC6473647F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBC6BB5D-D41F-3F41-BCA0-546B442281B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="620" windowWidth="51200" windowHeight="26960" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trade_1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="87">
   <si>
     <t>TradeId</t>
   </si>
@@ -278,16 +278,13 @@
     <t>InterestRateSwap</t>
   </si>
   <si>
-    <t>FXForward</t>
+    <t>FxOption</t>
+  </si>
+  <si>
+    <t>CrossCurrencySwap</t>
   </si>
   <si>
     <t>FxForward</t>
-  </si>
-  <si>
-    <t>FxOption</t>
-  </si>
-  <si>
-    <t>CrossCurrencySwap</t>
   </si>
 </sst>
 </file>
@@ -836,7 +833,7 @@
         <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -862,7 +859,7 @@
         <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
@@ -933,7 +930,7 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -968,7 +965,7 @@
         <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
@@ -1072,7 +1069,7 @@
         <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -1131,7 +1128,7 @@
         <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>

</xml_diff>